<commit_message>
fixed correction 05/05/2026 22:55
</commit_message>
<xml_diff>
--- a/SMI-Excels/TR/TR-DOMSC.xlsx
+++ b/SMI-Excels/TR/TR-DOMSC.xlsx
@@ -1,41 +1,155 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\DEC\SMI-Excels\TR\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7351441-D344-46D6-9119-B2AAE68F6BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="1060" yWindow="1060" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
+  <si>
+    <t>PeriodDec</t>
+  </si>
+  <si>
+    <t>NbrEcritures</t>
+  </si>
+  <si>
+    <t>Agence</t>
+  </si>
+  <si>
+    <t>TypeIdentifiant</t>
+  </si>
+  <si>
+    <t>CodeIdentifiant</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Prenom</t>
+  </si>
+  <si>
+    <t>Nationalite</t>
+  </si>
+  <si>
+    <t>CategBenif</t>
+  </si>
+  <si>
+    <t>AnneScol</t>
+  </si>
+  <si>
+    <t>DatDebScol</t>
+  </si>
+  <si>
+    <t>DatFinScol</t>
+  </si>
+  <si>
+    <t>NumDomDosScol</t>
+  </si>
+  <si>
+    <t>DatDomDosScol</t>
+  </si>
+  <si>
+    <t>OuvRenDosScol</t>
+  </si>
+  <si>
+    <t>DatOuvRen</t>
+  </si>
+  <si>
+    <t>NumAutBCT</t>
+  </si>
+  <si>
+    <t>DateAutBCT</t>
+  </si>
+  <si>
+    <t>BoursEtude</t>
+  </si>
+  <si>
+    <t>MntBoursDev</t>
+  </si>
+  <si>
+    <t>CodDevMntBourse</t>
+  </si>
+  <si>
+    <t>MntBoursTnd</t>
+  </si>
+  <si>
+    <t>DureBours</t>
+  </si>
+  <si>
+    <t>DatDebBours</t>
+  </si>
+  <si>
+    <t>DatFinBours</t>
+  </si>
+  <si>
+    <t>DatClotDosScolIat</t>
+  </si>
+  <si>
+    <t>CodIATClot</t>
+  </si>
+  <si>
+    <t>CodPaysDest</t>
+  </si>
+  <si>
+    <t>012026</t>
+  </si>
+  <si>
+    <t>000001</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>12345678</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>2025-2026</t>
+  </si>
+  <si>
+    <t>15/03/2026</t>
+  </si>
+  <si>
+    <t>1234567890123</t>
+  </si>
+  <si>
+    <t>AUTO-123</t>
+  </si>
+  <si>
+    <t>788</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +179,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,155 +518,156 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>PeriodDec</v>
-      </c>
-      <c r="B1" t="str">
-        <v>NbrEcritures</v>
-      </c>
-      <c r="C1" t="str">
-        <v>PeriodDec</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Agence</v>
-      </c>
-      <c r="E1" t="str">
-        <v>TypeIdentifiant</v>
-      </c>
-      <c r="F1" t="str">
-        <v>CodeIdentifiant</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Nom</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Prenom</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Nationalite</v>
-      </c>
-      <c r="J1" t="str">
-        <v>CategBenif</v>
-      </c>
-      <c r="K1" t="str">
-        <v>AnneScol</v>
-      </c>
-      <c r="L1" t="str">
-        <v>DatDebScol</v>
-      </c>
-      <c r="M1" t="str">
-        <v>DatFinScol</v>
-      </c>
-      <c r="N1" t="str">
-        <v>NumDomDosScol</v>
-      </c>
-      <c r="O1" t="str">
-        <v>DatDomDosScol</v>
-      </c>
-      <c r="P1" t="str">
-        <v>OuvRenDosScol</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>DatOuvRen</v>
-      </c>
-      <c r="R1" t="str">
-        <v>NumAutBCT</v>
-      </c>
-      <c r="S1" t="str">
-        <v>DateAutBCT</v>
-      </c>
-      <c r="T1" t="str">
-        <v>BoursEtude</v>
-      </c>
-      <c r="U1" t="str">
-        <v>MntBoursDev</v>
-      </c>
-      <c r="V1" t="str">
-        <v>CodDevMntBourse</v>
-      </c>
-      <c r="W1" t="str">
-        <v>MntBoursTnd</v>
-      </c>
-      <c r="X1" t="str">
-        <v>DureBours</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>DatDebBours</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>DatFinBours</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>DatClotDosScolIat</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>CodIATClot</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>CodPaysDest</v>
+    <row r="1" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>012026</v>
-      </c>
-      <c r="B2" t="str">
-        <v>000001</v>
-      </c>
-      <c r="C2" t="str">
-        <v>012026</v>
-      </c>
-      <c r="D2" t="str">
-        <v>023</v>
-      </c>
-      <c r="E2" t="str">
-        <v>C</v>
-      </c>
-      <c r="F2" t="str">
-        <v>12345678</v>
-      </c>
-      <c r="G2" t="str">
-        <v>TEST</v>
-      </c>
-      <c r="H2" t="str">
-        <v>TEST</v>
-      </c>
-      <c r="I2" t="str">
-        <v>123</v>
+    <row r="2" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>33</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
-      <c r="K2" t="str">
-        <v>2025-2026</v>
-      </c>
-      <c r="L2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="M2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="N2" t="str">
-        <v>1234567890123</v>
-      </c>
-      <c r="O2" t="str">
-        <v>15/03/2026</v>
+      <c r="K2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" t="s">
+        <v>35</v>
       </c>
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="R2" t="str">
-        <v>AUTO-123</v>
-      </c>
-      <c r="S2" t="str">
-        <v>15/03/2026</v>
+      <c r="Q2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" t="s">
+        <v>35</v>
       </c>
       <c r="T2">
         <v>1</v>
@@ -552,34 +675,35 @@
       <c r="U2">
         <v>1000</v>
       </c>
-      <c r="V2" t="str">
-        <v>788</v>
+      <c r="V2" t="s">
+        <v>38</v>
       </c>
       <c r="W2">
         <v>1000</v>
       </c>
-      <c r="X2" t="str">
-        <v>12</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>15/03/2026</v>
-      </c>
-      <c r="AB2" t="str">
-        <v>02</v>
-      </c>
-      <c r="AC2" t="str">
-        <v>123</v>
+      <c r="X2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError sqref="A1:AC1 A2:C2 E2:AC2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>